<commit_message>
Fixed errors in patient_clusters file
</commit_message>
<xml_diff>
--- a/results/cluster_analysis/survival_diseasefree_analysis/survival_diseasefree_statistical_tests.xlsx
+++ b/results/cluster_analysis/survival_diseasefree_analysis/survival_diseasefree_statistical_tests.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlos Paja Suarez\Desktop\imo_clustering\results\cluster_analysis\survival_diseasefree_analysis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlos Paja Suarez\imoc_pdac\results\cluster_analysis\survival_diseasefree_analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{304583E1-790A-4E4D-AC71-1D5781CB1D3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C0280F8-410B-43E3-A726-BFB91E3D63C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{63B67F03-D473-4F89-8E09-F2B6EC80F7B5}"/>
   </bookViews>
   <sheets>
     <sheet name="summary of all tests" sheetId="1" r:id="rId1"/>
+    <sheet name="tables_figures" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="184">
   <si>
     <t>overall</t>
   </si>
@@ -361,13 +362,238 @@
   </si>
   <si>
     <t>N (p=0.022)</t>
+  </si>
+  <si>
+    <t>Restricted mean survival time (p-value)</t>
+  </si>
+  <si>
+    <t>Hazard ratio</t>
+  </si>
+  <si>
+    <t>0.216</t>
+  </si>
+  <si>
+    <t>0.152</t>
+  </si>
+  <si>
+    <t>0.122</t>
+  </si>
+  <si>
+    <t>0.064</t>
+  </si>
+  <si>
+    <t>0.050</t>
+  </si>
+  <si>
+    <t>0.056</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>% patients disease free</t>
+  </si>
+  <si>
+    <t>1/27/59</t>
+  </si>
+  <si>
+    <t>7/24/56</t>
+  </si>
+  <si>
+    <t>12/22/53</t>
+  </si>
+  <si>
+    <t>20/18/49</t>
+  </si>
+  <si>
+    <t>40/12/35</t>
+  </si>
+  <si>
+    <t>64/5/18</t>
+  </si>
+  <si>
+    <t>Cluster 2, at risk/censored/recurrence</t>
+  </si>
+  <si>
+    <t>0/12/14</t>
+  </si>
+  <si>
+    <t>1/12/13</t>
+  </si>
+  <si>
+    <t>4/11/11</t>
+  </si>
+  <si>
+    <t>7/10/9</t>
+  </si>
+  <si>
+    <t>16/5/5</t>
+  </si>
+  <si>
+    <t>23/2/1</t>
+  </si>
+  <si>
+    <t>Cluster 1, at risk/censored/recurrence</t>
+  </si>
+  <si>
+    <t>Overall</t>
+  </si>
+  <si>
+    <t>18 months</t>
+  </si>
+  <si>
+    <t>6 months</t>
+  </si>
+  <si>
+    <t>DISEASE-FREE TABLE</t>
+  </si>
+  <si>
+    <t>1.57</t>
+  </si>
+  <si>
+    <t>1.49</t>
+  </si>
+  <si>
+    <t>0.070</t>
+  </si>
+  <si>
+    <t>% patients alive</t>
+  </si>
+  <si>
+    <t>3/42/76</t>
+  </si>
+  <si>
+    <t>10/39/72</t>
+  </si>
+  <si>
+    <t>21/33/67</t>
+  </si>
+  <si>
+    <t>39/26/56</t>
+  </si>
+  <si>
+    <t>73/14/34</t>
+  </si>
+  <si>
+    <t>98/5/18</t>
+  </si>
+  <si>
+    <t>Cluster 2, at risk/censored/death events</t>
+  </si>
+  <si>
+    <t>1/18/14</t>
+  </si>
+  <si>
+    <t>2/17/14</t>
+  </si>
+  <si>
+    <t>5/14/14</t>
+  </si>
+  <si>
+    <t>12/13/8</t>
+  </si>
+  <si>
+    <t>22/6/5</t>
+  </si>
+  <si>
+    <t>30/2/1</t>
+  </si>
+  <si>
+    <t>Cluster 1, at risk/censored/death events</t>
+  </si>
+  <si>
+    <t>SURVIVAL TABLE</t>
+  </si>
+  <si>
+    <t>0.34 (0.047)</t>
+  </si>
+  <si>
+    <t>1.49 (0.012)</t>
+  </si>
+  <si>
+    <t>2.66 (0.018)</t>
+  </si>
+  <si>
+    <t>3.53 (0.038)</t>
+  </si>
+  <si>
+    <t>4.56 (0.113)</t>
+  </si>
+  <si>
+    <t>2.23 (0.571)</t>
+  </si>
+  <si>
+    <t>0.37 (&lt;0.01)</t>
+  </si>
+  <si>
+    <t>1.06 (0.013)</t>
+  </si>
+  <si>
+    <t>1.92 (0.031)</t>
+  </si>
+  <si>
+    <t>2.48 (0.067)</t>
+  </si>
+  <si>
+    <t>3.32 (0.192)</t>
+  </si>
+  <si>
+    <t>7.72 (0.144)</t>
+  </si>
+  <si>
+    <t>11.62 (0.097)</t>
+  </si>
+  <si>
+    <t>Heinze log-rank test p-value</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>1.85 (0.646)</t>
+  </si>
+  <si>
+    <t>87</t>
+  </si>
+  <si>
+    <t>71</t>
+  </si>
+  <si>
+    <t>44</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>82</t>
+  </si>
+  <si>
+    <t>58</t>
+  </si>
+  <si>
+    <t>32</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -388,6 +614,20 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -422,7 +662,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -430,11 +670,283 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="19">
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -445,6 +957,40 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9105EAF7-DB9F-4E91-8265-9745B6C46770}" name="Tabla1" displayName="Tabla1" ref="A2:H8" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
+  <autoFilter ref="A2:H8" xr:uid="{9105EAF7-DB9F-4E91-8265-9745B6C46770}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{78B41C5F-8552-4217-B024-2FAED3CCE920}" name=" " dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{F9877DA9-8CB3-44FA-8F7A-59BD30FD8CF1}" name="6 months" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{AD27E9F3-F9CD-4CAC-8BEF-CE0D780EF708}" name="1 year" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{0CA6424F-DE76-40E4-9CD0-749FF0B2F21C}" name="18 months" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{0484B256-8F55-40B6-9FCC-501BE88A3AAB}" name="2 years" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{ED2CB652-B7FB-43FA-A41F-5A27F82573FA}" name="3 years" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{D08BC632-6277-43FC-9F8B-C456F3986032}" name="5 years" dataDxfId="10"/>
+    <tableColumn id="8" xr3:uid="{03D568A4-1271-4222-953C-5B6DD6FD7B9F}" name="Overall" dataDxfId="9"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{24602037-8553-4109-928B-9B19CD0209B5}" name="Tabla2" displayName="Tabla2" ref="A12:H18" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A12:H18" xr:uid="{24602037-8553-4109-928B-9B19CD0209B5}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{018D9221-1012-456D-8622-5C241903C431}" name=" " dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{0A2DEBAA-D4BC-4780-B634-BEC3ABDB4464}" name="6 months" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{35143CBE-D729-45C2-9CB7-DA9DD4E6C11C}" name="1 year"/>
+    <tableColumn id="4" xr3:uid="{F278BE74-980A-4AD0-BF4E-DEC044B1A28D}" name="18 months" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{1B11DD86-0739-40ED-BCEC-075CFF93A10A}" name="2 years" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{B0FC9546-8B22-40FF-B33E-999AD7403229}" name="3 years" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{A32D6658-D29B-4B46-AE8B-E2DE542C5132}" name="5 years" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{433013EC-9750-4DE5-9716-296B8EF94E42}" name="Overall" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1181,4 +1727,395 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F0893BD-D1BD-4F92-BDE6-BFF200B3959B}">
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="35" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="11" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="C6" s="8">
+        <v>0.13400000000000001</v>
+      </c>
+      <c r="D6" s="8">
+        <v>5.6000000000000001E-2</v>
+      </c>
+      <c r="E6" s="8">
+        <v>0.316</v>
+      </c>
+      <c r="F6" s="8">
+        <v>0.20499999999999999</v>
+      </c>
+      <c r="G6" s="8">
+        <v>0.11700000000000001</v>
+      </c>
+      <c r="H6" s="8">
+        <v>0.113</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="B7" s="8">
+        <v>4.6399999999999997</v>
+      </c>
+      <c r="C7" s="8">
+        <v>1.92</v>
+      </c>
+      <c r="D7" s="8">
+        <v>2.0699999999999998</v>
+      </c>
+      <c r="E7" s="8">
+        <v>1.41</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="G7" s="8">
+        <v>1.54</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="7" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" s="13" t="s">
+        <v>170</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="H13" s="8" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="H14" s="8" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="H15" s="8" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="H16" s="8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>110</v>
+      </c>
+      <c r="B17" s="12">
+        <v>5.67</v>
+      </c>
+      <c r="C17" s="12">
+        <v>2.4300000000000002</v>
+      </c>
+      <c r="D17" s="12">
+        <v>1.91</v>
+      </c>
+      <c r="E17" s="12">
+        <v>1.69</v>
+      </c>
+      <c r="F17" s="12">
+        <v>1.52</v>
+      </c>
+      <c r="G17" s="12">
+        <v>1.42</v>
+      </c>
+      <c r="H17" s="12">
+        <v>1.42</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="H18" s="8" t="s">
+        <v>171</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="2">
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>